<commit_message>
Enable reviewed government announcement sources
</commit_message>
<xml_diff>
--- a/sources.xlsx
+++ b/sources.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R05211df233594d82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rb9b807859d5a4d0a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2520,24 +2520,264 @@
       </x:c>
     </x:row>
     <x:row r="62">
-      <x:c r="A62"/>
-      <x:c r="B62"/>
-      <x:c r="C62"/>
-      <x:c r="D62"/>
-      <x:c r="E62"/>
-      <x:c r="F62"/>
-      <x:c r="G62"/>
-      <x:c r="H62"/>
+      <x:c r="A62" t="str">
+        <x:v>国家能源局—通知</x:v>
+      </x:c>
+      <x:c r="B62" t="str">
+        <x:v>政府机构</x:v>
+      </x:c>
+      <x:c r="C62" t="str">
+        <x:v>综合新能源</x:v>
+      </x:c>
+      <x:c r="D62" t="str">
+        <x:v>能源政策/通知</x:v>
+      </x:c>
+      <x:c r="E62" t="str">
+        <x:v>工作日</x:v>
+      </x:c>
+      <x:c r="F62" t="str">
+        <x:v>国家能源局发布的能源政策通知、工作安排和监管文件。</x:v>
+      </x:c>
+      <x:c r="G62" t="str">
+        <x:v>官方公开栏目；固定 HTTPS/同域路径；仅抓取机关文件纯文本；不下载附件、图片、音视频或政策解读。</x:v>
+      </x:c>
+      <x:c r="H62" t="str">
+        <x:v>https://www.nea.gov.cn/policy/tz.htm</x:v>
+      </x:c>
     </x:row>
     <x:row r="63">
-      <x:c r="A63"/>
-      <x:c r="B63"/>
-      <x:c r="C63"/>
-      <x:c r="D63"/>
-      <x:c r="E63"/>
-      <x:c r="F63"/>
-      <x:c r="G63"/>
-      <x:c r="H63"/>
+      <x:c r="A63" t="str">
+        <x:v>国家能源局—公告</x:v>
+      </x:c>
+      <x:c r="B63" t="str">
+        <x:v>政府机构</x:v>
+      </x:c>
+      <x:c r="C63" t="str">
+        <x:v>综合新能源</x:v>
+      </x:c>
+      <x:c r="D63" t="str">
+        <x:v>能源政策/公告</x:v>
+      </x:c>
+      <x:c r="E63" t="str">
+        <x:v>工作日</x:v>
+      </x:c>
+      <x:c r="F63" t="str">
+        <x:v>国家能源局发布的行政公告和行业监管公告。</x:v>
+      </x:c>
+      <x:c r="G63" t="str">
+        <x:v>官方公开栏目；固定 HTTPS/同域路径；仅抓取机关文件纯文本；不下载附件、图片、音视频或政策解读。</x:v>
+      </x:c>
+      <x:c r="H63" t="str">
+        <x:v>https://www.nea.gov.cn/policy/gg.htm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" t="str">
+        <x:v>工业和信息化部—文件公示</x:v>
+      </x:c>
+      <x:c r="B64" t="str">
+        <x:v>政府机构</x:v>
+      </x:c>
+      <x:c r="C64" t="str">
+        <x:v>综合科技</x:v>
+      </x:c>
+      <x:c r="D64" t="str">
+        <x:v>产业政策/公示</x:v>
+      </x:c>
+      <x:c r="E64" t="str">
+        <x:v>工作日</x:v>
+      </x:c>
+      <x:c r="F64" t="str">
+        <x:v>工业和信息化部文件公示，覆盖产业、装备、制造业和信息化监管动态。</x:v>
+      </x:c>
+      <x:c r="G64" t="str">
+        <x:v>官方公开栏目；固定 HTTPS/同域路径；仅抓取机关公示纯文本；不下载附件、图片、音视频或政策解读。</x:v>
+      </x:c>
+      <x:c r="H64" t="str">
+        <x:v>https://www.miit.gov.cn/zwgk/wjgs/index.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" t="str">
+        <x:v>科学技术部—通知通告</x:v>
+      </x:c>
+      <x:c r="B65" t="str">
+        <x:v>政府机构</x:v>
+      </x:c>
+      <x:c r="C65" t="str">
+        <x:v>综合科技</x:v>
+      </x:c>
+      <x:c r="D65" t="str">
+        <x:v>科技政策/通知</x:v>
+      </x:c>
+      <x:c r="E65" t="str">
+        <x:v>工作日</x:v>
+      </x:c>
+      <x:c r="F65" t="str">
+        <x:v>科学技术部发布的科研项目、科技管理和政策通知。</x:v>
+      </x:c>
+      <x:c r="G65" t="str">
+        <x:v>官方公开栏目；固定 HTTPS/同域路径；仅抓取机关通知纯文本；不下载附件、图片、音视频或政策解读。</x:v>
+      </x:c>
+      <x:c r="H65" t="str">
+        <x:v>https://www.most.gov.cn/tztg/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" t="str">
+        <x:v>自然资源部—通知公告</x:v>
+      </x:c>
+      <x:c r="B66" t="str">
+        <x:v>政府机构</x:v>
+      </x:c>
+      <x:c r="C66" t="str">
+        <x:v>综合新能源</x:v>
+      </x:c>
+      <x:c r="D66" t="str">
+        <x:v>自然资源政策/通知公告</x:v>
+      </x:c>
+      <x:c r="E66" t="str">
+        <x:v>工作日</x:v>
+      </x:c>
+      <x:c r="F66" t="str">
+        <x:v>自然资源部发布的自然资源管理通知公告。</x:v>
+      </x:c>
+      <x:c r="G66" t="str">
+        <x:v>官方公开栏目；当前仅保存标题、日期和官方原文链接，不请求详情正文。</x:v>
+      </x:c>
+      <x:c r="H66" t="str">
+        <x:v>https://www.mnr.gov.cn/gk/tzgg/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" t="str">
+        <x:v>交通运输部—其他政策性文件</x:v>
+      </x:c>
+      <x:c r="B67" t="str">
+        <x:v>政府机构</x:v>
+      </x:c>
+      <x:c r="C67" t="str">
+        <x:v>综合科技</x:v>
+      </x:c>
+      <x:c r="D67" t="str">
+        <x:v>交通政策/文件</x:v>
+      </x:c>
+      <x:c r="E67" t="str">
+        <x:v>工作日</x:v>
+      </x:c>
+      <x:c r="F67" t="str">
+        <x:v>交通运输部发布的其他政策性文件，覆盖交通产业、运输管理和技术政策。</x:v>
+      </x:c>
+      <x:c r="G67" t="str">
+        <x:v>官方公开栏目；固定 HTTPS/同域路径；仅抓取机关文件纯文本；不下载附件、图片、音视频或政策解读。</x:v>
+      </x:c>
+      <x:c r="H67" t="str">
+        <x:v>https://xxgk.mot.gov.cn/2020/zhengce/qtwjlist.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" t="str">
+        <x:v>商务部—政策发布</x:v>
+      </x:c>
+      <x:c r="B68" t="str">
+        <x:v>政府机构</x:v>
+      </x:c>
+      <x:c r="C68" t="str">
+        <x:v>综合科技</x:v>
+      </x:c>
+      <x:c r="D68" t="str">
+        <x:v>商务政策/文件</x:v>
+      </x:c>
+      <x:c r="E68" t="str">
+        <x:v>工作日</x:v>
+      </x:c>
+      <x:c r="F68" t="str">
+        <x:v>商务部政策发布，覆盖贸易、投资、流通和产业政策。</x:v>
+      </x:c>
+      <x:c r="G68" t="str">
+        <x:v>官方公开栏目；仅限 /zcfb/ 机关文件；排除政策解读；不下载附件、图片或音视频。</x:v>
+      </x:c>
+      <x:c r="H68" t="str">
+        <x:v>https://www.mofcom.gov.cn/zcfb/index.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" t="str">
+        <x:v>应急管理部—通知公告</x:v>
+      </x:c>
+      <x:c r="B69" t="str">
+        <x:v>政府机构</x:v>
+      </x:c>
+      <x:c r="C69" t="str">
+        <x:v>综合科技</x:v>
+      </x:c>
+      <x:c r="D69" t="str">
+        <x:v>安全应急/通知公告</x:v>
+      </x:c>
+      <x:c r="E69" t="str">
+        <x:v>工作日</x:v>
+      </x:c>
+      <x:c r="F69" t="str">
+        <x:v>应急管理部发布的安全生产、应急管理和防灾减灾通知公告。</x:v>
+      </x:c>
+      <x:c r="G69" t="str">
+        <x:v>官方公开栏目；固定 HTTPS/同域路径；仅抓取机关文件纯文本；不下载附件、图片、音视频或政策解读。</x:v>
+      </x:c>
+      <x:c r="H69" t="str">
+        <x:v>https://www.mem.gov.cn/gk/tzgg/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" t="str">
+        <x:v>国家数据局—政策发布</x:v>
+      </x:c>
+      <x:c r="B70" t="str">
+        <x:v>政府机构</x:v>
+      </x:c>
+      <x:c r="C70" t="str">
+        <x:v>综合科技</x:v>
+      </x:c>
+      <x:c r="D70" t="str">
+        <x:v>数据政策/文件</x:v>
+      </x:c>
+      <x:c r="E70" t="str">
+        <x:v>工作日</x:v>
+      </x:c>
+      <x:c r="F70" t="str">
+        <x:v>国家数据局发布的数据基础制度、数字经济和数据要素政策。</x:v>
+      </x:c>
+      <x:c r="G70" t="str">
+        <x:v>官方公开栏目；仅限 /zcfb/ 主记录；排除图解和专家解读；不下载附件、图片或音视频。</x:v>
+      </x:c>
+      <x:c r="H70" t="str">
+        <x:v>https://www.nda.gov.cn/sjj/zwgk/zcfb/list/index_pc_1.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" t="str">
+        <x:v>市场监管总局—反垄断通知公告</x:v>
+      </x:c>
+      <x:c r="B71" t="str">
+        <x:v>政府机构</x:v>
+      </x:c>
+      <x:c r="C71" t="str">
+        <x:v>综合科技</x:v>
+      </x:c>
+      <x:c r="D71" t="str">
+        <x:v>市场监管/反垄断</x:v>
+      </x:c>
+      <x:c r="E71" t="str">
+        <x:v>工作日</x:v>
+      </x:c>
+      <x:c r="F71" t="str">
+        <x:v>国家市场监督管理总局反垄断通知公告。</x:v>
+      </x:c>
+      <x:c r="G71" t="str">
+        <x:v>官方公开栏目；固定 HTTPS/同域路径；仅抓取机关公告纯文本；不下载附件、图片、音视频或政策解读。</x:v>
+      </x:c>
+      <x:c r="H71" t="str">
+        <x:v>https://www.samr.gov.cn/jzxts/tzgg/index.html</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: track NCSTI artificial intelligence news
</commit_message>
<xml_diff>
--- a/sources.xlsx
+++ b/sources.xlsx
@@ -320,7 +320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H77"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.80000019073486"/>
   <cols>
     <col width="32.5546875" customWidth="1" min="1" max="1"/>
@@ -3503,6 +3503,48 @@
         </is>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>北京国际科技创新中心—人工智能热点</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>政府科技资讯平台</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>AI与智能科技</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>人工智能科技热点</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>工作日</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>北京国际科技创新中心网络服务平台人工智能科技热点栏目，追踪人工智能技术、科研与产业动态。</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>官方栏目；限定该栏目日期正文；包含科技日报等转载稿，按原文链接去重。</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>https://www.ncsti.gov.cn/kjdt/kjrd/rgzn_kjrd/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: track NCSTI artificial intelligence news (#46)
</commit_message>
<xml_diff>
--- a/sources.xlsx
+++ b/sources.xlsx
@@ -320,7 +320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H77"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.80000019073486"/>
   <cols>
     <col width="32.5546875" customWidth="1" min="1" max="1"/>
@@ -3503,6 +3503,48 @@
         </is>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>北京国际科技创新中心—人工智能热点</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>政府科技资讯平台</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>AI与智能科技</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>人工智能科技热点</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>工作日</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>北京国际科技创新中心网络服务平台人工智能科技热点栏目，追踪人工智能技术、科研与产业动态。</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>官方栏目；限定该栏目日期正文；包含科技日报等转载稿，按原文链接去重。</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>https://www.ncsti.gov.cn/kjdt/kjrd/rgzn_kjrd/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: track academic frontier and archive conference calendars monthly
</commit_message>
<xml_diff>
--- a/sources.xlsx
+++ b/sources.xlsx
@@ -320,7 +320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.80000019073486"/>
   <cols>
     <col width="32.5546875" customWidth="1" min="1" max="1"/>
@@ -3545,6 +3545,48 @@
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>mtl.inew.cn—学术前沿</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>学术资讯网站</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>综合科技</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>学术前沿</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>工作日</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>mtl.inew.cn 学术前沿栏目，追踪研究进展与科研动态。</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>栏目链接；本环境域名连接超时，页面结构尚待真实站点验证；抓取失败须记录为失败而非零新闻。</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>https://mtl.inew.cn/academic-news/frontier?lang=zh</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: track academic frontier and archive conference calendars monthly (#47)
</commit_message>
<xml_diff>
--- a/sources.xlsx
+++ b/sources.xlsx
@@ -320,7 +320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.80000019073486"/>
   <cols>
     <col width="32.5546875" customWidth="1" min="1" max="1"/>
@@ -3545,6 +3545,48 @@
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>mtl.inew.cn—学术前沿</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>学术资讯网站</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>综合科技</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>学术前沿</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>工作日</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>mtl.inew.cn 学术前沿栏目，追踪研究进展与科研动态。</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>栏目链接；本环境域名连接超时，页面结构尚待真实站点验证；抓取失败须记录为失败而非零新闻。</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>https://mtl.inew.cn/academic-news/frontier?lang=zh</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>